<commit_message>
latest 2026-09-01 export image
</commit_message>
<xml_diff>
--- a/数据导出/discovery_rules.xlsx
+++ b/数据导出/discovery_rules.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,6 +539,117 @@
       </c>
       <c r="I3" s="1" t="n">
         <v>46129.37647059297</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Network interface discovery</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>net.if.discovery[node_exporter]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>91001</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>46261.35537078948</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>46261.35537078948</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Block devices discovery</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>vfs.dev.discovery[node_exporter]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>91001</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>46261.35537078948</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>46261.35537078948</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mounted filesystem discovery</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>vfs.fs.discovery[node_exporter]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>91001</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>46261.35537078948</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>46261.35537078948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>